<commit_message>
release: prepare v1.0.0 public release
</commit_message>
<xml_diff>
--- a/economics/Economic_Assessment_Group3.xlsx
+++ b/economics/Economic_Assessment_Group3.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="106">
   <si>
     <t xml:space="preserve">Economic Assessment — Group 3 geothermal binary plant</t>
   </si>
@@ -73,6 +73,15 @@
     <t xml:space="preserve">from ORC_Group3.xlsx &gt; Base_Case_Group3!B17</t>
   </si>
   <si>
+    <t xml:space="preserve">Average Production Temperature (°C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">°C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validated FEFLOW post-processing output (Stage 12), t = 100 yr; see ../outputs/Average_Production_Temperature.csv, ../figures/F8_average_production_temperature.png</t>
+  </si>
+  <si>
     <t xml:space="preserve">UNIT COSTS (from Xodo lecture, Zero-Emission Binary CAPEX table)</t>
   </si>
   <si>
@@ -98,6 +107,9 @@
   </si>
   <si>
     <t xml:space="preserve">€/m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scaled from Xodo reference example (2,500 m, &gt;250 degC); linear depth-scaling assumption applied to Group 3 (1,120 m wells)</t>
   </si>
   <si>
     <t xml:space="preserve">Long production testing</t>
@@ -337,11 +349,11 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="12">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="#,##0&quot; €&quot;"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="#,##0&quot; €/kW&quot;"/>
-    <numFmt numFmtId="168" formatCode="#,##0&quot; kW&quot;"/>
-    <numFmt numFmtId="169" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="#,##0&quot; €&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="#,##0&quot; €/kW&quot;"/>
+    <numFmt numFmtId="169" formatCode="#,##0&quot; kW&quot;"/>
     <numFmt numFmtId="170" formatCode="#,##0&quot; €/kW-yr&quot;"/>
     <numFmt numFmtId="171" formatCode="#,##0&quot; h/yr&quot;"/>
     <numFmt numFmtId="172" formatCode="#,##0.0&quot; €/MWh&quot;"/>
@@ -349,7 +361,7 @@
     <numFmt numFmtId="174" formatCode="0%"/>
     <numFmt numFmtId="175" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -408,13 +420,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -487,96 +492,100 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -656,7 +665,6 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
-  <c:style val="2"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -671,14 +679,14 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr sz="1800" b="1" u="none" strike="noStrike">
+              <a:rPr lang="en-US" sz="1800" b="1" u="none" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>LCOE Sensitivity — Spider Diagram (Group 3)</a:t>
+              <a:t> LCOE Spider Diagram </a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -701,7 +709,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sensitivity!C4</c:f>
+              <c:f>Sensitivity!$C$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -732,36 +740,31 @@
           </c:marker>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
-            <c:showLeaderLines val="1"/>
-            <c:leaderLines>
-              <c:spPr>
-                <a:ln w="12600">
-                  <a:solidFill>
-                    <a:srgbClr val="000000"/>
-                  </a:solidFill>
-                </a:ln>
-              </c:spPr>
-            </c:leaderLines>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
+                <c15:showLeaderLines val="0"/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -795,19 +798,19 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>291.670975006444</c:v>
+                  <c:v>294.205381211103</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>226.314914675121</c:v>
+                  <c:v>228.030966631161</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>185.274075135268</c:v>
+                  <c:v>186.521696718949</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>157.569955272</c:v>
+                  <c:v>158.525671343925</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>137.86753657404</c:v>
+                  <c:v>138.625693697318</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -819,7 +822,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sensitivity!E4</c:f>
+              <c:f>Sensitivity!$E$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -850,36 +853,31 @@
           </c:marker>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
-            <c:showLeaderLines val="1"/>
-            <c:leaderLines>
-              <c:spPr>
-                <a:ln w="12600">
-                  <a:solidFill>
-                    <a:srgbClr val="000000"/>
-                  </a:solidFill>
-                </a:ln>
-              </c:spPr>
-            </c:leaderLines>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
+                <c15:showLeaderLines val="0"/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -913,19 +911,19 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>177.790007925684</c:v>
+                  <c:v>178.907854076065</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>181.085139999594</c:v>
+                  <c:v>182.259925240325</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>185.274075135268</c:v>
+                  <c:v>186.521696718949</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>190.487444881876</c:v>
+                  <c:v>191.832547542768</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>196.906585470638</c:v>
+                  <c:v>198.374651581898</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -937,7 +935,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sensitivity!G4</c:f>
+              <c:f>Sensitivity!$G$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -968,36 +966,31 @@
           </c:marker>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
-            <c:showLeaderLines val="1"/>
-            <c:leaderLines>
-              <c:spPr>
-                <a:ln w="12600">
-                  <a:solidFill>
-                    <a:srgbClr val="000000"/>
-                  </a:solidFill>
-                </a:ln>
-              </c:spPr>
-            </c:leaderLines>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
+                <c15:showLeaderLines val="0"/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -1031,19 +1024,19 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>220.04003480769</c:v>
+                  <c:v>221.601571266304</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>200.725612767455</c:v>
+                  <c:v>202.113645175113</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>185.274075135268</c:v>
+                  <c:v>186.521696718949</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>172.631907981659</c:v>
+                  <c:v>173.767570860652</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>162.096768686986</c:v>
+                  <c:v>163.137792992729</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1055,7 +1048,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sensitivity!I4</c:f>
+              <c:f>Sensitivity!$I$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1086,36 +1079,31 @@
           </c:marker>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
-            <c:showLeaderLines val="1"/>
-            <c:leaderLines>
-              <c:spPr>
-                <a:ln w="12600">
-                  <a:solidFill>
-                    <a:srgbClr val="000000"/>
-                  </a:solidFill>
-                </a:ln>
-              </c:spPr>
-            </c:leaderLines>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
+                <c15:showLeaderLines val="0"/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -1149,19 +1137,19 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>168.953365512434</c:v>
+                  <c:v>170.055983549665</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>177.113720323851</c:v>
+                  <c:v>178.289643925912</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>185.274075135268</c:v>
+                  <c:v>186.521696718949</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>193.434429946684</c:v>
+                  <c:v>194.756964678406</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>201.594784758101</c:v>
+                  <c:v>202.990625054653</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1173,7 +1161,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sensitivity!K4</c:f>
+              <c:f>Sensitivity!$K$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1204,36 +1192,31 @@
           </c:marker>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
-            <c:showLeaderLines val="1"/>
-            <c:leaderLines>
-              <c:spPr>
-                <a:ln w="12600">
-                  <a:solidFill>
-                    <a:srgbClr val="000000"/>
-                  </a:solidFill>
-                </a:ln>
-              </c:spPr>
-            </c:leaderLines>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
+                <c15:showLeaderLines val="0"/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -1267,19 +1250,19 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>168.953365512434</c:v>
+                  <c:v>170.055983549665</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>177.113720323851</c:v>
+                  <c:v>178.289643925912</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>185.274075135268</c:v>
+                  <c:v>186.521696718949</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>193.434429946684</c:v>
+                  <c:v>194.756964678406</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>201.594784758101</c:v>
+                  <c:v>202.990625054653</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1294,51 +1277,18 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="89615472"/>
-        <c:axId val="94215449"/>
+        <c:axId val="47898974"/>
+        <c:axId val="46132162"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="89615472"/>
+        <c:axId val="47898974"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="0"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
-                    <a:uFillTx/>
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr sz="1000" b="1" u="none" strike="noStrike">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:uFillTx/>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
-                  <a:t>Variation from base case</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln w="0">
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-        </c:title>
-        <c:numFmt formatCode="0%" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:numFmt formatCode="0%" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -1364,7 +1314,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94215449"/>
+        <c:crossAx val="46132162"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1372,57 +1322,14 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="94215449"/>
+        <c:axId val="46132162"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9360">
-              <a:solidFill>
-                <a:srgbClr val="878787"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
-                    <a:uFillTx/>
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr sz="1000" b="1" u="none" strike="noStrike">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:uFillTx/>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
-                  <a:t>LCOE [€/MWh]</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln w="0">
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-        </c:title>
-        <c:numFmt formatCode="0.0" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -1448,7 +1355,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89615472"/>
+        <c:crossAx val="47898974"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1730,9 +1637,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>448200</xdr:colOff>
+      <xdr:colOff>447480</xdr:colOff>
       <xdr:row>32</xdr:row>
-      <xdr:rowOff>149760</xdr:rowOff>
+      <xdr:rowOff>149040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1740,8 +1647,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="2300760"/>
-        <a:ext cx="7919640" cy="3959640"/>
+        <a:off x="0" y="2200320"/>
+        <a:ext cx="7918920" cy="3768480"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1935,388 +1842,398 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D34"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="55"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="D6" s="3"/>
+    </row>
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <f aca="false">B5+B6</f>
         <v>10</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="D7" s="3"/>
+    </row>
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="5" t="n">
         <v>1120</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="4" t="n">
-        <v>4261.8</v>
-      </c>
-      <c r="C10" s="0" t="s">
+      <c r="B10" s="5" t="n">
+        <v>4223.9</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="B11" s="6" t="n">
+        <v>124.5327</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="D11" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="5" t="n">
         <v>20000</v>
       </c>
-      <c r="C13" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="4" t="n">
+      <c r="C13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="3"/>
+    </row>
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="5" t="n">
         <v>700000</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="3"/>
+    </row>
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>400000</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="3"/>
+    </row>
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>2200</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" s="3"/>
+    </row>
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" s="3"/>
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" s="3"/>
+    </row>
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>750000</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D20" s="3"/>
+    </row>
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>400000</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="3"/>
+    </row>
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D22" s="3"/>
+    </row>
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" s="3"/>
+    </row>
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D26" s="3"/>
+    </row>
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+    </row>
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D28" s="3"/>
+    </row>
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B29" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="D14" s="2"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>400000</v>
-      </c>
-      <c r="C15" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>2200</v>
-      </c>
-      <c r="C16" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="2" t="e">
-        <f aca="false">5,500,0 € / 2,500 m (Xodo example well)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="B17" s="4" t="n">
-        <v>500000</v>
-      </c>
-      <c r="C17" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="D17" s="2"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="C18" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="2"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>500000</v>
-      </c>
-      <c r="C19" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="D19" s="2"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" s="4" t="n">
-        <v>750000</v>
-      </c>
-      <c r="C20" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="D20" s="2"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="B21" s="4" t="n">
-        <v>400000</v>
-      </c>
-      <c r="C21" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" s="2"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" s="4" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="C22" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="D22" s="2"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="B23" s="4" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="C23" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="D23" s="2"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="B24" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="C24" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="B25" s="4" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C25" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D26" s="2"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="B28" s="4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C28" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="D28" s="2"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="C29" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D29" s="3"/>
+    </row>
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B29" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="C29" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="D29" s="2"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="B30" s="4" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="C30" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="B31" s="0" t="n">
+      <c r="D30" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B31" s="1" t="n">
         <f aca="false">B30*8760</f>
         <v>8322</v>
       </c>
-      <c r="C31" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="D31" s="2"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="B32" s="4" t="n">
+      <c r="C31" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D31" s="3"/>
+    </row>
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="C32" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="D32" s="2"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="B33" s="4" t="n">
+      <c r="C32" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D32" s="3"/>
+    </row>
+    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C33" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="B34" s="0" t="n">
+      <c r="C33" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="1" t="n">
         <f aca="false">B28*(1+B28)^B29/((1+B28)^B29-1)</f>
         <v>0.117459624772546</v>
       </c>
-      <c r="C34" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>56</v>
+      <c r="C34" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -2341,332 +2258,332 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" s="0" t="n">
+    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" s="1" t="n">
         <f aca="false">Assumptions!B10/(1-Assumptions!B25)/1000</f>
-        <v>5.01388235294118</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E6" s="6" t="s">
+        <v>4.96929411764706</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="B6" s="8" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="C6" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B7" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="0" t="n">
+      <c r="D6" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="1" t="n">
         <f aca="false">Assumptions!B24</f>
         <v>10</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="9" t="n">
         <f aca="false">Assumptions!B13</f>
         <v>20000</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="9" t="n">
         <f aca="false">C7*D7</f>
         <v>200000</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="10" t="n">
         <f aca="false">E7/$E$18</f>
-        <v>0.00384484033735081</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="B8" s="0" t="s">
+        <v>0.0038514430450868</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="0" t="n">
+      <c r="C8" s="1" t="n">
         <f aca="false">Assumptions!B8</f>
         <v>2</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="9" t="n">
         <f aca="false">Assumptions!B14</f>
         <v>700000</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="9" t="n">
         <f aca="false">C8*D8</f>
         <v>1400000</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="10" t="n">
         <f aca="false">E8/$E$18</f>
-        <v>0.0269138823614557</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="0" t="s">
+        <v>0.0269601013156076</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="0" t="n">
+      <c r="C9" s="1" t="n">
         <f aca="false">Assumptions!B7</f>
         <v>10</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="9" t="n">
         <f aca="false">Assumptions!B15</f>
         <v>400000</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="9" t="n">
         <f aca="false">C9*D9</f>
         <v>4000000</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="10" t="n">
         <f aca="false">E9/$E$18</f>
-        <v>0.0768968067470163</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="C10" s="0" t="n">
+        <v>0.0770288609017361</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10" s="1" t="n">
         <f aca="false">Assumptions!B7*Assumptions!B9</f>
         <v>11200</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="9" t="n">
         <f aca="false">Assumptions!B16</f>
         <v>2200</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E10" s="9" t="n">
         <f aca="false">C10*D10</f>
         <v>24640000</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="10" t="n">
         <f aca="false">E10/$E$18</f>
-        <v>0.47368432956162</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="C11" s="0" t="n">
+        <v>0.474497783154694</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="9" t="n">
         <f aca="false">Assumptions!B17</f>
         <v>500000</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="9" t="n">
         <f aca="false">C11*D11</f>
         <v>500000</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="10" t="n">
         <f aca="false">E11/$E$18</f>
-        <v>0.00961210084337704</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>72</v>
-      </c>
-      <c r="B12" s="0" t="s">
-        <v>73</v>
-      </c>
-      <c r="C12" s="0" t="n">
+        <v>0.00962860761271701</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="1" t="n">
         <f aca="false">B4</f>
-        <v>5.01388235294118</v>
-      </c>
-      <c r="D12" s="7" t="n">
+        <v>4.96929411764706</v>
+      </c>
+      <c r="D12" s="9" t="n">
         <f aca="false">Assumptions!B18</f>
         <v>2000000</v>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="E12" s="9" t="n">
         <f aca="false">C12*D12</f>
-        <v>10027764.7058824</v>
-      </c>
-      <c r="F12" s="8" t="n">
+        <v>9938588.23529412</v>
+      </c>
+      <c r="F12" s="10" t="n">
         <f aca="false">E12/$E$18</f>
-        <v>0.192775771173197</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>74</v>
-      </c>
-      <c r="B13" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="C13" s="0" t="n">
+        <v>0.191389532684025</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="9" t="n">
         <f aca="false">Assumptions!B19</f>
         <v>500000</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="E13" s="9" t="n">
         <f aca="false">C13*D13</f>
         <v>500000</v>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="F13" s="10" t="n">
         <f aca="false">E13/$E$18</f>
-        <v>0.00961210084337704</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+        <v>0.00962860761271701</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B14" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="C14" s="0" t="n">
+      <c r="C14" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="9" t="n">
         <f aca="false">Assumptions!B20</f>
         <v>750000</v>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="E14" s="9" t="n">
         <f aca="false">C14*D14</f>
         <v>750000</v>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="F14" s="10" t="n">
         <f aca="false">E14/$E$18</f>
-        <v>0.0144181512650656</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>76</v>
-      </c>
-      <c r="B15" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="C15" s="0" t="n">
+        <v>0.0144429114190755</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" s="1" t="n">
         <f aca="false">Assumptions!B5</f>
         <v>5</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="9" t="n">
         <f aca="false">Assumptions!B21</f>
         <v>400000</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="9" t="n">
         <f aca="false">C15*D15</f>
         <v>2000000</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="F15" s="10" t="n">
         <f aca="false">E15/$E$18</f>
-        <v>0.0384484033735081</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="B16" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="C16" s="0" t="n">
+        <v>0.0385144304508681</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="1" t="n">
         <f aca="false">Assumptions!B8</f>
         <v>2</v>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="9" t="n">
         <f aca="false">Assumptions!B22</f>
         <v>3000000</v>
       </c>
-      <c r="E16" s="7" t="n">
+      <c r="E16" s="9" t="n">
         <f aca="false">C16*D16</f>
         <v>6000000</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F16" s="10" t="n">
         <f aca="false">E16/$E$18</f>
-        <v>0.115345210120524</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="B17" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="C17" s="0" t="n">
+        <v>0.115543291352604</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="9" t="n">
         <f aca="false">Assumptions!B23</f>
         <v>2000000</v>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="E17" s="9" t="n">
         <f aca="false">C17*D17</f>
         <v>2000000</v>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="F17" s="10" t="n">
         <f aca="false">E17/$E$18</f>
-        <v>0.0384484033735081</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="12" t="n">
+        <v>0.0385144304508681</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="14" t="n">
         <f aca="false">SUM(E7:E17)</f>
-        <v>52017764.7058824</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B20" s="13" t="n">
+        <v>51928588.2352941</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B20" s="15" t="n">
         <f aca="false">E18/Assumptions!B10</f>
-        <v>12205.5855990151</v>
+        <v>12293.9909172315</v>
       </c>
     </row>
   </sheetData>
@@ -2686,92 +2603,92 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="B4" s="7" t="n">
+    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="9" t="n">
         <f aca="false">CAPEX_Group3!E18</f>
-        <v>52017764.7058824</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="B5" s="14" t="n">
+        <v>51928588.2352941</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" s="16" t="n">
         <f aca="false">Assumptions!B10</f>
-        <v>4261.8</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="B6" s="13" t="n">
+        <v>4223.9</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="15" t="n">
         <f aca="false">B4/B5</f>
-        <v>12205.5855990151</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="15" t="n">
+        <v>12293.9909172315</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" s="6" t="n">
         <f aca="false">Assumptions!B34</f>
         <v>0.117459624772546</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="B8" s="16" t="n">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="17" t="n">
         <f aca="false">Assumptions!B33</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="B9" s="17" t="n">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="18" t="n">
         <f aca="false">Assumptions!B31</f>
         <v>8322</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="B10" s="18" t="n">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" s="19" t="n">
         <f aca="false">Assumptions!B32</f>
         <v>13</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="B12" s="20" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="21" t="n">
         <f aca="false">(B6*B7+B8)/B9*1000+B10</f>
-        <v>185.273913072518</v>
+        <v>186.521696718949</v>
       </c>
     </row>
   </sheetData>
@@ -2791,264 +2708,269 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="15"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="C4" s="6" t="s">
+    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D4" s="6" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="E4" s="6" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="B4" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="D4" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="E4" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="F4" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="G4" s="8" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="n">
+      <c r="H4" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="22" t="n">
         <v>-0.2</v>
       </c>
-      <c r="B5" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="C5" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((100)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((100)-(50))/LN((273.15+(100))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((100)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((100)-(50))/LN((273.15+(100))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>291.670975006444</v>
-      </c>
-      <c r="D5" s="0" t="n">
+      <c r="B5" s="1" t="n">
+        <f aca="false">Assumptions!$B$11*(1+A5)</f>
+        <v>99.62616</v>
+      </c>
+      <c r="C5" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((B5)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((B5)-(50))/LN((273.15+(B5))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((B5)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((B5)-(50))/LN((273.15+(B5))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>294.205381211103</v>
+      </c>
+      <c r="D5" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="E5" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(40)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(40))/LN((273.15+(125))/(273.15+(40)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(40)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(40))/LN((273.15+(125))/(273.15+(40)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>177.790007925684</v>
-      </c>
-      <c r="F5" s="0" t="n">
+      <c r="E5" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((Assumptions!$B$11)-(40)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(40))/LN((273.15+(Assumptions!$B$11))/(273.15+(40)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((Assumptions!$B$11)-(40)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(40))/LN((273.15+(Assumptions!$B$11))/(273.15+(40)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>178.907854076065</v>
+      </c>
+      <c r="F5" s="1" t="n">
         <v>120</v>
       </c>
-      <c r="G5" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((120)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((120)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>220.04003480769</v>
-      </c>
-      <c r="H5" s="0" t="n">
+      <c r="G5" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((120)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((120)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>221.601571266304</v>
+      </c>
+      <c r="H5" s="1" t="n">
         <v>896</v>
       </c>
-      <c r="I5" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(896)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>168.953365512434</v>
-      </c>
-      <c r="J5" s="0" t="n">
+      <c r="I5" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(896)*10)+(2000000*(((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>170.055983549665</v>
+      </c>
+      <c r="J5" s="1" t="n">
         <v>1760</v>
       </c>
-      <c r="K5" s="22" t="n">
-        <f aca="false">(((17350000+((1760)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>168.953365512434</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="n">
+      <c r="K5" s="23" t="n">
+        <f aca="false">(((17350000+((1760)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>170.055983549665</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="22" t="n">
         <v>-0.1</v>
       </c>
-      <c r="B6" s="0" t="n">
-        <v>112.5</v>
-      </c>
-      <c r="C6" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((112.5)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((112.5)-(50))/LN((273.15+(112.5))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((112.5)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((112.5)-(50))/LN((273.15+(112.5))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>226.314914675121</v>
-      </c>
-      <c r="D6" s="0" t="n">
+      <c r="B6" s="1" t="n">
+        <f aca="false">Assumptions!$B$11*(1+A6)</f>
+        <v>112.07943</v>
+      </c>
+      <c r="C6" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((B6)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((B6)-(50))/LN((273.15+(B6))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((B6)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((B6)-(50))/LN((273.15+(B6))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>228.030966631161</v>
+      </c>
+      <c r="D6" s="1" t="n">
         <v>45</v>
       </c>
-      <c r="E6" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(45)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(45))/LN((273.15+(125))/(273.15+(45)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(45)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(45))/LN((273.15+(125))/(273.15+(45)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>181.085139999594</v>
-      </c>
-      <c r="F6" s="0" t="n">
+      <c r="E6" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((Assumptions!$B$11)-(45)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(45))/LN((273.15+(Assumptions!$B$11))/(273.15+(45)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((Assumptions!$B$11)-(45)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(45))/LN((273.15+(Assumptions!$B$11))/(273.15+(45)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>182.259925240325</v>
+      </c>
+      <c r="F6" s="1" t="n">
         <v>135</v>
       </c>
-      <c r="G6" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((135)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((135)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>200.725612767455</v>
-      </c>
-      <c r="H6" s="0" t="n">
+      <c r="G6" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((135)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((135)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>202.113645175113</v>
+      </c>
+      <c r="H6" s="1" t="n">
         <v>1008</v>
       </c>
-      <c r="I6" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1008)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>177.113720323851</v>
-      </c>
-      <c r="J6" s="0" t="n">
+      <c r="I6" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1008)*10)+(2000000*(((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>178.289643925912</v>
+      </c>
+      <c r="J6" s="1" t="n">
         <v>1980</v>
       </c>
-      <c r="K6" s="22" t="n">
-        <f aca="false">(((17350000+((1980)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>177.113720323851</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="n">
+      <c r="K6" s="23" t="n">
+        <f aca="false">(((17350000+((1980)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>178.289643925912</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="B7" s="0" t="n">
-        <v>125</v>
-      </c>
-      <c r="C7" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>185.274075135268</v>
-      </c>
-      <c r="D7" s="0" t="n">
+      <c r="B7" s="6" t="n">
+        <f aca="false">Assumptions!$B$11</f>
+        <v>124.5327</v>
+      </c>
+      <c r="C7" s="23" t="n">
+        <f aca="false">LCOE_Group3!$B$12</f>
+        <v>186.521696718949</v>
+      </c>
+      <c r="D7" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="E7" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>185.274075135268</v>
-      </c>
-      <c r="F7" s="0" t="n">
+      <c r="E7" s="23" t="n">
+        <f aca="false">LCOE_Group3!$B$12</f>
+        <v>186.521696718949</v>
+      </c>
+      <c r="F7" s="1" t="n">
         <v>150</v>
       </c>
-      <c r="G7" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>185.274075135268</v>
-      </c>
-      <c r="H7" s="0" t="n">
+      <c r="G7" s="23" t="n">
+        <f aca="false">LCOE_Group3!$B$12</f>
+        <v>186.521696718949</v>
+      </c>
+      <c r="H7" s="1" t="n">
         <v>1120</v>
       </c>
-      <c r="I7" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>185.274075135268</v>
-      </c>
-      <c r="J7" s="0" t="n">
+      <c r="I7" s="23" t="n">
+        <f aca="false">LCOE_Group3!$B$12</f>
+        <v>186.521696718949</v>
+      </c>
+      <c r="J7" s="1" t="n">
         <v>2200</v>
       </c>
-      <c r="K7" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>185.274075135268</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="n">
+      <c r="K7" s="23" t="n">
+        <f aca="false">LCOE_Group3!$B$12</f>
+        <v>186.521696718949</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="22" t="n">
         <v>0.1</v>
       </c>
-      <c r="B8" s="0" t="n">
-        <v>137.5</v>
-      </c>
-      <c r="C8" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((137.5)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((137.5)-(50))/LN((273.15+(137.5))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((137.5)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((137.5)-(50))/LN((273.15+(137.5))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>157.569955272</v>
-      </c>
-      <c r="D8" s="0" t="n">
+      <c r="B8" s="1" t="n">
+        <f aca="false">Assumptions!$B$11*(1+A8)</f>
+        <v>136.98597</v>
+      </c>
+      <c r="C8" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((B8)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((B8)-(50))/LN((273.15+(B8))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((B8)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((B8)-(50))/LN((273.15+(B8))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>158.525671343925</v>
+      </c>
+      <c r="D8" s="1" t="n">
         <v>55</v>
       </c>
-      <c r="E8" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(55)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(55))/LN((273.15+(125))/(273.15+(55)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(55)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(55))/LN((273.15+(125))/(273.15+(55)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>190.487444881876</v>
-      </c>
-      <c r="F8" s="0" t="n">
+      <c r="E8" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((Assumptions!$B$11)-(55)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(55))/LN((273.15+(Assumptions!$B$11))/(273.15+(55)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((Assumptions!$B$11)-(55)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(55))/LN((273.15+(Assumptions!$B$11))/(273.15+(55)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>191.832547542768</v>
+      </c>
+      <c r="F8" s="1" t="n">
         <v>165</v>
       </c>
-      <c r="G8" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((165)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((165)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>172.631907981659</v>
-      </c>
-      <c r="H8" s="0" t="n">
+      <c r="G8" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((165)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((165)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>173.767570860652</v>
+      </c>
+      <c r="H8" s="1" t="n">
         <v>1232</v>
       </c>
-      <c r="I8" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1232)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>193.434429946684</v>
-      </c>
-      <c r="J8" s="0" t="n">
+      <c r="I8" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1232)*10)+(2000000*(((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>194.756964678406</v>
+      </c>
+      <c r="J8" s="1" t="n">
         <v>2420</v>
       </c>
-      <c r="K8" s="22" t="n">
-        <f aca="false">(((17350000+((2420)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>193.434429946684</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="n">
+      <c r="K8" s="23" t="n">
+        <f aca="false">(((17350000+((2420)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>194.756964678406</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="22" t="n">
         <v>0.2</v>
       </c>
-      <c r="B9" s="0" t="n">
-        <v>150</v>
-      </c>
-      <c r="C9" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((150)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((150)-(50))/LN((273.15+(150))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((150)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((150)-(50))/LN((273.15+(150))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>137.86753657404</v>
-      </c>
-      <c r="D9" s="0" t="n">
+      <c r="B9" s="1" t="n">
+        <f aca="false">Assumptions!$B$11*(1+A9)</f>
+        <v>149.43924</v>
+      </c>
+      <c r="C9" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((B9)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((B9)-(50))/LN((273.15+(B9))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((B9)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((B9)-(50))/LN((273.15+(B9))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>138.625693697318</v>
+      </c>
+      <c r="D9" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="E9" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(60)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(60))/LN((273.15+(125))/(273.15+(60)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(60)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(60))/LN((273.15+(125))/(273.15+(60)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>196.906585470638</v>
-      </c>
-      <c r="F9" s="0" t="n">
+      <c r="E9" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((Assumptions!$B$11)-(60)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(60))/LN((273.15+(Assumptions!$B$11))/(273.15+(60)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((Assumptions!$B$11)-(60)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(60))/LN((273.15+(Assumptions!$B$11))/(273.15+(60)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>198.374651581898</v>
+      </c>
+      <c r="F9" s="1" t="n">
         <v>180</v>
       </c>
-      <c r="G9" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((180)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((180)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>162.096768686986</v>
-      </c>
-      <c r="H9" s="0" t="n">
+      <c r="G9" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1120)*10)+(2000000*(((((180)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((180)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>163.137792992729</v>
+      </c>
+      <c r="H9" s="1" t="n">
         <v>1344</v>
       </c>
-      <c r="I9" s="22" t="n">
-        <f aca="false">(((17350000+((2200)*(1344)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>201.594784758101</v>
-      </c>
-      <c r="J9" s="0" t="n">
+      <c r="I9" s="23" t="n">
+        <f aca="false">(((17350000+((2200)*(1344)*10)+(2000000*(((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>202.990625054653</v>
+      </c>
+      <c r="J9" s="1" t="n">
         <v>2640</v>
       </c>
-      <c r="K9" s="22" t="n">
-        <f aca="false">(((17350000+((2640)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((125)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((125)-(50))/LN((273.15+(125))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
-        <v>201.594784758101</v>
+      <c r="K9" s="23" t="n">
+        <f aca="false">(((17350000+((2640)*(1120)*10)+(2000000*(((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15)))))/0.85/1000)))/((((150)*0.917)*4.31*((Assumptions!$B$11)-(50)))*(0.52*(1-(273.15+19.9590607511086)/(273.15+(((Assumptions!$B$11)-(50))/LN((273.15+(Assumptions!$B$11))/(273.15+(50)))-273.15))))))*0.117459624772546)/8322*1000+13</f>
+        <v>202.990625054653</v>
       </c>
     </row>
   </sheetData>

</xml_diff>